<commit_message>
IV infusion time for PFOA was set to 0.003 h (10.8 s), instead of using a bolus, so initial distribution will be the same with 1 or 2 blood compartments.
</commit_message>
<xml_diff>
--- a/Inputs/PFOA_template_parameters_Exposure.xlsx
+++ b/Inputs/PFOA_template_parameters_Exposure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="496" documentId="14_{BC2287C1-70F4-4BAE-BA85-F3EC3C708A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DD6B41E-5F49-4854-9791-ABDA2AFAD1DD}"/>
+  <xr:revisionPtr revIDLastSave="497" documentId="14_{BC2287C1-70F4-4BAE-BA85-F3EC3C708A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCA93E98-637E-4BAF-803E-D724DECDE5E0}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="19770" windowHeight="14130" tabRatio="668" activeTab="4" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="2595" yWindow="2460" windowWidth="25740" windowHeight="12795" tabRatio="668" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="MKudo1BW" sheetId="40" r:id="rId1"/>
@@ -1092,6 +1092,9 @@
       <c r="C23" t="s">
         <v>24</v>
       </c>
+      <c r="E23">
+        <v>3.0000000000000001E-3</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
@@ -3390,11 +3393,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3867,7 +3865,21 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
@@ -3912,24 +3924,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E78C79C6-E5CC-4F2D-A2E3-1FF685DFF167}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3952,7 +3947,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3965,12 +3976,4 @@
     <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Reset PFOA Kudo1 exposure to be bolus IV, not infusion.
</commit_message>
<xml_diff>
--- a/Inputs/PFOA_template_parameters_Exposure.xlsx
+++ b/Inputs/PFOA_template_parameters_Exposure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="497" documentId="14_{BC2287C1-70F4-4BAE-BA85-F3EC3C708A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCA93E98-637E-4BAF-803E-D724DECDE5E0}"/>
+  <xr:revisionPtr revIDLastSave="500" documentId="14_{BC2287C1-70F4-4BAE-BA85-F3EC3C708A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14F1A6FD-4130-4F60-BDBB-B8F2496398BD}"/>
   <bookViews>
-    <workbookView xWindow="2595" yWindow="2460" windowWidth="25740" windowHeight="12795" tabRatio="668" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="1513" yWindow="1667" windowWidth="21600" windowHeight="12586" tabRatio="668" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="MKudo1BW" sheetId="40" r:id="rId1"/>
@@ -438,10 +438,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -741,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D69B4C24-1AC5-42FA-88F9-A86A51928A45}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -982,7 +978,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>90</v>
       </c>
@@ -996,7 +992,7 @@
         <v>82.057366080959994</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>93</v>
       </c>
@@ -1013,7 +1009,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>97</v>
       </c>
@@ -1030,7 +1026,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
@@ -1047,7 +1043,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1061,7 +1057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1082,7 +1078,7 @@
         <v>4.1000000000000002E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>53</v>
       </c>
@@ -1092,11 +1088,15 @@
       <c r="C23" t="s">
         <v>24</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23">
+        <f>F23*60*60</f>
+        <v>10.799999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>12</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>15</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>108</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>64</v>
       </c>
@@ -1171,7 +1171,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>65</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>67</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -3393,6 +3393,65 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3865,66 +3924,38 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E78C79C6-E5CC-4F2D-A2E3-1FF685DFF167}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3945,35 +3976,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>